<commit_message>
fable-r2d2: final package - 9/9 slice check, 99-page manual and full verification
- every part slices on the H2D with no warnings: 10,053.9 g and 320.6 h for twelve pieces
- 99-page illustrated manual, 33 figures embedded, every page rendered
- bill-of-materials spreadsheet refreshed with the final print figures
- scripts/verify.py ALL PASS: images, cad, bom, wiring, firmware, audio, drawings, manual, video
</commit_message>
<xml_diff>
--- a/fable-r2d2/bom/bill-of-materials.xlsx
+++ b/fable-r2d2/bom/bill-of-materials.xlsx
@@ -5075,10 +5075,10 @@
         <v>1304.3</v>
       </c>
       <c r="I2" s="8" t="n">
-        <v>1243.9</v>
+        <v>1243.4</v>
       </c>
       <c r="J2" s="8" t="n">
-        <v>35.37</v>
+        <v>35.36</v>
       </c>
       <c r="K2" s="9" t="inlineStr">
         <is>
@@ -5120,13 +5120,13 @@
         <v>264</v>
       </c>
       <c r="H3" s="8" t="n">
-        <v>3325.6</v>
+        <v>3445.3</v>
       </c>
       <c r="I3" s="8" t="n">
-        <v>0</v>
+        <v>3115.1</v>
       </c>
       <c r="J3" s="8" t="n">
-        <v>0</v>
+        <v>107.62</v>
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
@@ -5168,13 +5168,13 @@
         <v>141.1</v>
       </c>
       <c r="H4" s="8" t="n">
-        <v>1952.2</v>
+        <v>2143.5</v>
       </c>
       <c r="I4" s="8" t="n">
-        <v>0</v>
+        <v>1939.4</v>
       </c>
       <c r="J4" s="8" t="n">
-        <v>0</v>
+        <v>59.24</v>
       </c>
       <c r="K4" s="9" t="inlineStr">
         <is>
@@ -5357,16 +5357,16 @@
         <v>100</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>47.518</v>
+        <v>34.292</v>
       </c>
       <c r="H8" s="8" t="n">
-        <v>326.6</v>
+        <v>246.8</v>
       </c>
       <c r="I8" s="8" t="n">
-        <v>162.3</v>
+        <v>128.3</v>
       </c>
       <c r="J8" s="8" t="n">
-        <v>5.42</v>
+        <v>4.25</v>
       </c>
       <c r="K8" s="9" t="inlineStr">
         <is>
@@ -5408,13 +5408,13 @@
         <v>119.9</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>489.8</v>
+        <v>510.1</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>322.4</v>
+        <v>330.7</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>9.16</v>
+        <v>9.48</v>
       </c>
       <c r="K9" s="9" t="inlineStr">
         <is>
@@ -5551,7 +5551,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5025.6</v>
+        <v>10053.9</v>
       </c>
       <c r="C2">
         <f>ROUNDUP(B2*1.25/1000,0)</f>

</xml_diff>

<commit_message>
fable-r2d2 revision D regeneration: bill of materials from the final mechanism and controls CSVs
</commit_message>
<xml_diff>
--- a/fable-r2d2/bom/bill-of-materials.xlsx
+++ b/fable-r2d2/bom/bill-of-materials.xlsx
@@ -6273,10 +6273,10 @@
         <v>3736.7</v>
       </c>
       <c r="I3" s="8" t="n">
-        <v>3285.2</v>
+        <v>3284.3</v>
       </c>
       <c r="J3" s="8" t="n">
-        <v>113.73</v>
+        <v>113.76</v>
       </c>
       <c r="K3" s="9" t="inlineStr">
         <is>
@@ -6420,7 +6420,7 @@
         <v>314.2</v>
       </c>
       <c r="J6" s="8" t="n">
-        <v>11.15</v>
+        <v>11.16</v>
       </c>
       <c r="K6" s="9" t="inlineStr">
         <is>
@@ -6561,7 +6561,7 @@
         <v>441.1</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>247.7</v>
+        <v>247.8</v>
       </c>
       <c r="J9" s="8" t="n">
         <v>7.9</v>
@@ -6749,7 +6749,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10598.4</v>
+        <v>10597.6</v>
       </c>
       <c r="C2">
         <f>ROUNDUP(B2*1.25/1000,0)</f>

</xml_diff>